<commit_message>
Further improvements to the example spec
</commit_message>
<xml_diff>
--- a/specs/ADSL_spec.xlsx
+++ b/specs/ADSL_spec.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t xml:space="preserve">Order</t>
   </si>
@@ -431,6 +431,60 @@
   </si>
   <si>
     <t xml:space="preserve">'Y' if DM.DTHDTC is not missing; otherwise 'N'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRTSDT = min(EX.EXSTDTC) as date, over EX records where EXDOSE &gt; 0 or (EXDOSE = 0 and EXTRT contains 'PLACEBO')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRTEDT = max(EX.EXENDTC) as date, over the same EX records used for TRTSDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRTDURD = TRTEDT - TRTSDT + 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGEGR1 = '&lt;65' if AGE &lt; 65; '65-80' if 65 &lt;= AGE &lt;= 80; '&gt;80' if AGE &gt; 80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAFFL = 'Y' if TRTSDT is not missing; else 'N'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOSSTT = 'COMPLETED' if DSDECOD = 'COMPLETED' for the DS record with DSCAT = 'DISPOSITION EVENT'; else 'DISCONTINUED'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOSDT = DS.DSSTDTC as date for the DS record with DSCAT = 'DISPOSITION EVENT'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DTHDT = DM.DTHDTC as date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DTHFL = 'Y' if DM.DTHDTC is not missing; else 'N'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First exposure date among treated EX records. Pseudo-code: TRTSDT = date(min(EX.EXSTDTC)) over EX records where EXDOSE &gt; 0 or (EXDOSE = 0 and EXTRT contains 'PLACEBO')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last exposure date among treated EX records. Pseudo-code: TRTEDT = date(max(EX.EXENDTC)) over the same EX records used for TRTSDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duration of treatment in days. Pseudo-code: TRTDURD = TRTEDT - TRTSDT + 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pool AGE into groups. Pseudo-code: AGEGR1 = '&lt;65' if AGE &lt; 65; '65-80' if 65 &lt;= AGE &lt;= 80; '&gt;80' if AGE &gt; 80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety population flag. Pseudo-code: SAFFL = 'Y' if TRTSDT is not missing, else 'N'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End of study status. Pseudo-code: EOSSTT = 'COMPLETED' if DSDECOD = 'COMPLETED' for the DS record with DSCAT = 'DISPOSITION EVENT', else 'DISCONTINUED'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End of study date. Pseudo-code: EOSDT = date(DS.DSSTDTC) for the DS record with DSCAT = 'DISPOSITION EVENT'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date of death. Pseudo-code: DTHDT = date(DM.DTHDTC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Death flag. Pseudo-code: DTHFL = 'Y' if DM.DTHDTC is not missing, else 'N'</t>
   </si>
 </sst>
 </file>
@@ -1412,7 +1466,9 @@
       <c r="F7" t="n">
         <v>8</v>
       </c>
-      <c r="G7"/>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
       <c r="H7"/>
       <c r="I7" t="s">
         <v>39</v>
@@ -1954,7 +2010,9 @@
       <c r="F19" t="n">
         <v>10</v>
       </c>
-      <c r="G19"/>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
       <c r="H19" t="s">
         <v>91</v>
       </c>
@@ -2001,7 +2059,9 @@
       <c r="F20" t="n">
         <v>10</v>
       </c>
-      <c r="G20"/>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
       <c r="H20" t="s">
         <v>91</v>
       </c>
@@ -2048,7 +2108,9 @@
       <c r="F21" t="n">
         <v>8</v>
       </c>
-      <c r="G21"/>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
       <c r="H21"/>
       <c r="I21" t="s">
         <v>39</v>
@@ -2138,7 +2200,9 @@
       <c r="F23" t="n">
         <v>10</v>
       </c>
-      <c r="G23"/>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
       <c r="H23" t="s">
         <v>91</v>
       </c>
@@ -2316,7 +2380,9 @@
       <c r="F27" t="n">
         <v>10</v>
       </c>
-      <c r="G27"/>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
       <c r="H27" t="s">
         <v>91</v>
       </c>
@@ -3564,10 +3630,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>First exposure date among treated EX records</t>
-        </is>
+      <c r="D2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="3">
@@ -3586,10 +3653,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Last exposure date among treated EX records</t>
-        </is>
+      <c r="D3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="4">
@@ -3608,10 +3676,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TRTEDT - TRTSDT + 1</t>
-        </is>
+      <c r="D4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F4" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="5">
@@ -3630,10 +3699,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Pool AGE into &lt;65 / 65-80 / &gt;80</t>
-        </is>
+      <c r="D5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F5" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="6">
@@ -3652,10 +3722,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Y if the subject has a non-missing TRTSDT, else N</t>
-        </is>
+      <c r="D6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F6" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="7">
@@ -3674,10 +3745,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Based on DS disposition event DSDECOD</t>
-        </is>
+      <c r="D7" t="s">
+        <v>150</v>
+      </c>
+      <c r="F7" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="8">
@@ -3696,10 +3768,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Based on DS disposition event DSSTDTC</t>
-        </is>
+      <c r="D8" t="s">
+        <v>151</v>
+      </c>
+      <c r="F8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="9">
@@ -3718,10 +3791,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>DM.DTHDTC converted to a date</t>
-        </is>
+      <c r="D9" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="10">
@@ -3740,10 +3814,11 @@
           <t>Computation</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Y if DM.DTHDTC is not missing, else N</t>
-        </is>
+      <c r="D10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>